<commit_message>
vault backup: 2026-05-03 17:30:27
</commit_message>
<xml_diff>
--- a/BWL/Übung/Übungen/UE05/BWL2T2_04_UE05_Kalkulation eines ... (Formular)_2022.xlsx
+++ b/BWL/Übung/Übungen/UE05/BWL2T2_04_UE05_Kalkulation eines ... (Formular)_2022.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t>BWL2T2</t>
   </si>
@@ -29,9 +29,6 @@
     <t xml:space="preserve">a) Ermittlung der Jahreskosten</t>
   </si>
   <si>
-    <t>Notes</t>
-  </si>
-  <si>
     <t xml:space="preserve">pro Monat</t>
   </si>
   <si>
@@ -42,9 +39,6 @@
   </si>
   <si>
     <t>1/6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Urlaubs- und Weihnachtsgeld</t>
   </si>
   <si>
     <t xml:space="preserve">Monatsentgelt (durchschnittlich)</t>
@@ -268,7 +262,7 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
@@ -298,6 +292,8 @@
     <xf fontId="0" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" quotePrefix="1"/>
     <xf fontId="0" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="4" borderId="0" numFmtId="3" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf fontId="0" fillId="4" borderId="0" numFmtId="10" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf fontId="0" fillId="4" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf fontId="0" fillId="4" borderId="1" numFmtId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -855,18 +851,15 @@
       <c r="A4" t="s">
         <v>2</v>
       </c>
-      <c r="H4" t="s">
-        <v>3</v>
-      </c>
     </row>
     <row r="5">
       <c r="F5" s="7" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F6" s="8">
         <v>3500</v>
@@ -874,11 +867,11 @@
     </row>
     <row r="7">
       <c r="A7" s="9" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" s="9"/>
       <c r="C7" s="10" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D7" s="11"/>
       <c r="E7" s="12"/>
@@ -886,13 +879,10 @@
         <f>F6/6</f>
         <v>583.33333333333337</v>
       </c>
-      <c r="H7" t="s">
-        <v>8</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F8" s="8">
         <f>SUM(F6:F7)</f>
@@ -901,7 +891,7 @@
     </row>
     <row r="9">
       <c r="A9" s="9" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B9" s="9"/>
       <c r="C9" s="14">
@@ -916,77 +906,77 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F10" s="8">
         <f>SUM(F8:F9)</f>
         <v>5308.3333333333339</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H10" s="1"/>
     </row>
     <row r="11">
       <c r="A11" s="16" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B11" s="16"/>
       <c r="C11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D11" s="8">
         <v>1200</v>
       </c>
       <c r="F11" s="8">
-        <f>D11/12</f>
+        <f t="shared" ref="F11:F12" si="0">D11/12</f>
         <v>100</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B12" s="9"/>
       <c r="C12" s="17" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D12" s="13">
         <v>1800</v>
       </c>
       <c r="E12" s="12"/>
       <c r="F12" s="13">
-        <f>D12/12</f>
+        <f t="shared" si="0"/>
         <v>150</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F13" s="8">
         <f>SUM(F10:F12)</f>
         <v>5558.3333333333339</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="16" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B15" s="16"/>
       <c r="C15" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D15" s="8">
         <f>200*12</f>
@@ -999,71 +989,71 @@
     </row>
     <row r="16">
       <c r="A16" s="16" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B16" s="16"/>
       <c r="C16" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D16" s="8">
         <v>1200</v>
       </c>
       <c r="E16" s="8"/>
       <c r="F16">
-        <f>D16/12</f>
+        <f t="shared" ref="F16:F17" si="1">D16/12</f>
         <v>100</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B17" s="9"/>
       <c r="C17" s="17" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D17" s="13">
         <v>2400</v>
       </c>
       <c r="E17" s="13"/>
       <c r="F17" s="12">
-        <f>D17/12</f>
+        <f t="shared" si="1"/>
         <v>200</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F18" s="8">
         <f>SUM(F15:F17)</f>
         <v>500</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F20" s="8">
         <f>F13+F18</f>
         <v>6058.3333333333339</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F21" s="1"/>
     </row>
     <row r="22">
       <c r="A22" s="9" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B22" s="9"/>
       <c r="C22" s="17"/>
@@ -1076,7 +1066,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F23" s="8">
         <f>F20+F22</f>
@@ -1085,36 +1075,36 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F24" s="18">
         <f>F23*12</f>
         <v>78516.000000000015</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="27">
       <c r="B27" t="s">
+        <v>31</v>
+      </c>
+      <c r="C27" t="s">
+        <v>32</v>
+      </c>
+      <c r="D27" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C27" t="s">
+      <c r="F27" t="s">
         <v>34</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="F27" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="28">
@@ -1123,131 +1113,201 @@
     </row>
     <row r="29">
       <c r="A29" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="B29" s="20"/>
-      <c r="C29" s="21"/>
-      <c r="D29" s="21"/>
-      <c r="F29" s="21"/>
+        <v>35</v>
+      </c>
+      <c r="B29" s="20">
+        <v>8</v>
+      </c>
+      <c r="C29" s="21">
+        <f>52*5</f>
+        <v>260</v>
+      </c>
+      <c r="D29" s="21">
+        <v>52</v>
+      </c>
+      <c r="F29" s="21">
+        <f>B29*C29</f>
+        <v>2080</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="16" t="s">
-        <v>38</v>
-      </c>
-      <c r="B30" s="20"/>
-      <c r="C30" s="21"/>
-      <c r="D30" s="21"/>
-      <c r="F30" s="21"/>
+        <v>36</v>
+      </c>
+      <c r="B30" s="20">
+        <v>8</v>
+      </c>
+      <c r="C30" s="21">
+        <v>25</v>
+      </c>
+      <c r="D30" s="21">
+        <v>5</v>
+      </c>
+      <c r="F30" s="21">
+        <f>B30*C30</f>
+        <v>200</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="B31" s="20"/>
-      <c r="C31" s="21"/>
-      <c r="D31" s="21"/>
-      <c r="F31" s="21"/>
+        <v>37</v>
+      </c>
+      <c r="B31" s="20">
+        <v>8</v>
+      </c>
+      <c r="C31" s="21">
+        <v>8</v>
+      </c>
+      <c r="D31" s="21">
+        <f>C31/5</f>
+        <v>1.6000000000000001</v>
+      </c>
+      <c r="F31" s="21">
+        <f>B31*C31</f>
+        <v>64</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="B32" s="22"/>
-      <c r="C32" s="23"/>
-      <c r="D32" s="23"/>
+        <v>38</v>
+      </c>
+      <c r="B32" s="22">
+        <v>8</v>
+      </c>
+      <c r="C32" s="23">
+        <v>10</v>
+      </c>
+      <c r="D32" s="23">
+        <v>2</v>
+      </c>
       <c r="E32" s="12"/>
-      <c r="F32" s="23"/>
+      <c r="F32" s="21">
+        <f>B32*C32</f>
+        <v>80</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>41</v>
-      </c>
-      <c r="F33" s="24"/>
+        <v>39</v>
+      </c>
+      <c r="F33" s="24">
+        <f>F29-(F30+F31+F32)</f>
+        <v>1736</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B34" s="9"/>
       <c r="C34" s="17"/>
       <c r="D34" s="12"/>
       <c r="E34" s="12"/>
-      <c r="F34" s="23"/>
+      <c r="F34" s="23">
+        <v>100</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
+        <v>41</v>
+      </c>
+      <c r="C35" t="s">
+        <v>42</v>
+      </c>
+      <c r="F35" s="24">
+        <f>F33-F34</f>
+        <v>1636</v>
+      </c>
+      <c r="G35" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="C35" t="s">
-        <v>44</v>
-      </c>
-      <c r="F35" s="24"/>
-      <c r="G35" s="2" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="37">
       <c r="C37" t="s">
-        <v>46</v>
-      </c>
-      <c r="E37" s="21"/>
+        <v>44</v>
+      </c>
+      <c r="E37" s="25">
+        <f>F35/F29</f>
+        <v>0.78653846153846152</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C38" t="s">
-        <v>48</v>
-      </c>
-      <c r="E38" s="8"/>
+        <v>46</v>
+      </c>
+      <c r="E38" s="21">
+        <f>F35/8</f>
+        <v>204.5</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>49</v>
-      </c>
-      <c r="F40" s="8"/>
+        <v>47</v>
+      </c>
+      <c r="F40" s="26">
+        <f>F24</f>
+        <v>78516.000000000015</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="16" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B41" s="16"/>
-      <c r="F41" s="25"/>
+      <c r="F41" s="27">
+        <f>F35</f>
+        <v>1636</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F42" s="8"/>
+        <v>50</v>
+      </c>
+      <c r="F42" s="8">
+        <f>F40/F41</f>
+        <v>47.992665036674822</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>53</v>
-      </c>
-      <c r="F43" s="8"/>
+        <v>51</v>
+      </c>
+      <c r="F43" s="8">
+        <f>F42*8</f>
+        <v>383.94132029339858</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F45" s="8"/>
+        <v>50</v>
+      </c>
+      <c r="F45" s="8">
+        <f>F10*12/F35</f>
+        <v>38.936430317848412</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>55</v>
-      </c>
-      <c r="F46" s="8"/>
+        <v>53</v>
+      </c>
+      <c r="F46" s="8">
+        <f>F45*8</f>
+        <v>311.4914425427873</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="75" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="74" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
 </worksheet>
 </file>

</xml_diff>